<commit_message>
Deployed 00a6476 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/CIEL1/CCF/CCF_2025/grille_comp_CCF.xlsx
+++ b/CIEL1/CCF/CCF_2025/grille_comp_CCF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\CIEL1\CCF\CCF_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED6D285-0067-4B83-87C8-8576CB9FDE5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7C61D4-F654-4728-91CD-8EBEECA766C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{5323A597-3EF7-45E9-BE64-C65DC6E6C1EB}"/>
   </bookViews>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="AQ3" s="1"/>
     </row>
-    <row r="4" spans="1:67" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:67" ht="17.649999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1255,20 +1255,42 @@
       <c r="V5">
         <v>0</v>
       </c>
-      <c r="W5" s="24"/>
-      <c r="X5"/>
+      <c r="W5" s="24">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
       <c r="Y5" s="28">
         <v>0</v>
       </c>
-      <c r="Z5" s="7"/>
-      <c r="AA5" s="35"/>
-      <c r="AB5" s="39"/>
-      <c r="AC5"/>
-      <c r="AD5" s="39"/>
-      <c r="AE5" s="7"/>
-      <c r="AF5" s="24"/>
-      <c r="AG5" s="35"/>
-      <c r="AH5" s="28"/>
+      <c r="Z5" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="39">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="28">
+        <v>0</v>
+      </c>
       <c r="AI5"/>
       <c r="AK5">
         <f>E5+P5+Z5+AE5</f>
@@ -1376,7 +1398,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="6" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6">
         <f>A5+1</f>
         <v>2</v>
@@ -1438,101 +1460,123 @@
       <c r="V6">
         <v>2</v>
       </c>
-      <c r="W6" s="24"/>
-      <c r="X6"/>
+      <c r="W6" s="24">
+        <v>2</v>
+      </c>
+      <c r="X6">
+        <v>2</v>
+      </c>
       <c r="Y6" s="28">
         <v>2</v>
       </c>
-      <c r="Z6" s="7"/>
-      <c r="AA6" s="35"/>
-      <c r="AB6" s="39"/>
-      <c r="AC6"/>
-      <c r="AD6" s="39"/>
-      <c r="AE6" s="7"/>
-      <c r="AF6" s="24"/>
-      <c r="AG6" s="35"/>
-      <c r="AH6" s="28"/>
+      <c r="Z6" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA6" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB6" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC6">
+        <v>2</v>
+      </c>
+      <c r="AD6" s="39">
+        <v>2</v>
+      </c>
+      <c r="AE6" s="7">
+        <v>2</v>
+      </c>
+      <c r="AF6" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="35">
+        <v>2</v>
+      </c>
+      <c r="AH6" s="28">
+        <v>2</v>
+      </c>
       <c r="AI6"/>
       <c r="AK6">
         <f t="shared" ref="AK6:AK32" si="5">E6+P6+Z6+AE6</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AL6">
         <f t="shared" ref="AL6:AL32" si="6">G6+M6+W6+AF6+J6</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AM6">
         <f t="shared" ref="AM6:AM32" si="7">F6+Q6+R6+AA6+AG6</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AN6">
         <f t="shared" ref="AN6:AN32" si="8">I6+N6+S6+U6+AB6+AD6</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AO6">
         <f t="shared" ref="AO6:AO32" si="9">K6+O6+T6+V6+X6+AC6</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AP6">
         <f t="shared" ref="AP6:AP32" si="10">H6+L6+Y6+AH6</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AR6">
         <f t="shared" ref="AR6:AR32" si="11">AK$2*AK6/(AK$3*2)</f>
-        <v>0.375</v>
+        <v>0.875</v>
       </c>
       <c r="AS6">
         <f t="shared" ref="AS6:AS32" si="12">AL$2*AL6/(AL$3*2)</f>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="AT6">
         <f t="shared" ref="AT6:AT32" si="13">AM$2*AM6/(AM$3*2)</f>
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="AU6">
         <f t="shared" ref="AU6:AU32" si="14">AN$2*AN6/(AN$3*2)</f>
-        <v>0.83333333333333337</v>
+        <v>1.5</v>
       </c>
       <c r="AV6">
         <f t="shared" ref="AV6:AV32" si="15">AO$2*AO6/(AO$3*2)</f>
-        <v>0.66666666666666663</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="AW6">
         <f t="shared" ref="AW6:AW32" si="16">AP$2*AP6/(AP$3*2)</f>
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="AY6" s="4">
         <f t="shared" ref="AY6:AY32" si="17">IF(AR6&gt;=0.75*AK$2, AK$2,AR6)</f>
-        <v>0.375</v>
+        <v>1</v>
       </c>
       <c r="AZ6" s="4">
         <f t="shared" ref="AZ6:AZ32" si="18">IF(AS6&gt;=0.75*AL$2, AL$2,AS6)</f>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BA6" s="4">
         <f t="shared" ref="BA6:BA32" si="19">IF(AT6&gt;=0.75*AM$2, AM$2,AT6)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BB6" s="4">
         <f t="shared" ref="BB6:BB32" si="20">IF(AU6&gt;=0.75*AN$2, AN$2,AU6)</f>
-        <v>0.83333333333333337</v>
+        <v>2</v>
       </c>
       <c r="BC6" s="4">
         <f t="shared" ref="BC6:BC32" si="21">IF(AV6&gt;=0.75*AO$2, AO$2,AV6)</f>
-        <v>0.66666666666666663</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="BD6" s="4">
         <f t="shared" ref="BD6:BD32" si="22">IF(AW6&gt;=0.75*AP$2, AP$2,AW6)</f>
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="BE6" s="4"/>
       <c r="BF6" s="2">
         <f t="shared" ref="BF6:BF32" si="23">SUM(AY6:BD6)</f>
-        <v>4.2249999999999996</v>
+        <v>8.3333333333333321</v>
       </c>
       <c r="BH6">
         <f t="shared" ref="BH6:BH32" si="24">ROUNDUP(AY6/0.5,0)*0.5</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI6">
         <f t="shared" ref="BI6:BI32" si="25">ROUNDUP(AZ6/0.5,0)*0.5</f>
@@ -1540,26 +1584,26 @@
       </c>
       <c r="BJ6">
         <f t="shared" ref="BJ6:BJ32" si="26">ROUNDUP(BA6/0.5,0)*0.5</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK6">
         <f t="shared" ref="BK6:BK32" si="27">ROUNDUP(BB6/0.5,0)*0.5</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BL6">
         <f t="shared" ref="BL6:BL32" si="28">ROUNDUP(BC6/0.5,0)*0.5</f>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BM6">
         <f t="shared" ref="BM6:BM32" si="29">ROUNDUP(BD6/0.5,0)*0.5</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BO6">
         <f t="shared" ref="BO6:BO32" si="30">SUM(BH6:BM6)</f>
-        <v>5.5</v>
+        <v>8.5</v>
       </c>
     </row>
-    <row r="7" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7">
         <f t="shared" ref="A7:A32" si="31">A6+1</f>
         <v>3</v>
@@ -1621,20 +1665,42 @@
       <c r="V7">
         <v>0</v>
       </c>
-      <c r="W7" s="24"/>
-      <c r="X7"/>
+      <c r="W7" s="24">
+        <v>2</v>
+      </c>
+      <c r="X7">
+        <v>2</v>
+      </c>
       <c r="Y7" s="28">
         <v>2</v>
       </c>
-      <c r="Z7" s="7"/>
-      <c r="AA7" s="35"/>
-      <c r="AB7" s="39"/>
-      <c r="AC7"/>
-      <c r="AD7" s="39"/>
-      <c r="AE7" s="7"/>
-      <c r="AF7" s="24"/>
-      <c r="AG7" s="35"/>
-      <c r="AH7" s="28"/>
+      <c r="Z7" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="39">
+        <v>1</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="28">
+        <v>0</v>
+      </c>
       <c r="AI7"/>
       <c r="AK7">
         <f t="shared" si="5"/>
@@ -1642,7 +1708,7 @@
       </c>
       <c r="AL7">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AM7">
         <f t="shared" si="7"/>
@@ -1650,11 +1716,11 @@
       </c>
       <c r="AN7">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO7">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP7">
         <f t="shared" si="10"/>
@@ -1666,7 +1732,7 @@
       </c>
       <c r="AS7">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="AT7">
         <f t="shared" si="13"/>
@@ -1674,11 +1740,11 @@
       </c>
       <c r="AU7">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="AV7">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AW7">
         <f t="shared" si="16"/>
@@ -1690,7 +1756,7 @@
       </c>
       <c r="AZ7" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="BA7" s="4">
         <f t="shared" si="19"/>
@@ -1698,11 +1764,11 @@
       </c>
       <c r="BB7" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="BC7" s="4">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="BD7" s="4">
         <f t="shared" si="22"/>
@@ -1711,7 +1777,7 @@
       <c r="BE7" s="4"/>
       <c r="BF7" s="2">
         <f t="shared" si="23"/>
-        <v>2.7583333333333333</v>
+        <v>3.6583333333333337</v>
       </c>
       <c r="BH7">
         <f t="shared" si="24"/>
@@ -1719,7 +1785,7 @@
       </c>
       <c r="BI7">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ7">
         <f t="shared" si="26"/>
@@ -1731,7 +1797,7 @@
       </c>
       <c r="BL7">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BM7">
         <f t="shared" si="29"/>
@@ -1739,10 +1805,10 @@
       </c>
       <c r="BO7">
         <f t="shared" si="30"/>
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
     </row>
-    <row r="8" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8">
         <f t="shared" si="31"/>
         <v>4</v>
@@ -1804,20 +1870,42 @@
       <c r="V8">
         <v>0</v>
       </c>
-      <c r="W8" s="24"/>
-      <c r="X8"/>
+      <c r="W8" s="24">
+        <v>1</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
       <c r="Y8" s="28">
         <v>0</v>
       </c>
-      <c r="Z8" s="7"/>
-      <c r="AA8" s="35"/>
-      <c r="AB8" s="39"/>
-      <c r="AC8"/>
-      <c r="AD8" s="39"/>
-      <c r="AE8" s="7"/>
-      <c r="AF8" s="24"/>
-      <c r="AG8" s="35"/>
-      <c r="AH8" s="28"/>
+      <c r="Z8" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="39">
+        <v>0</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="28">
+        <v>0</v>
+      </c>
       <c r="AI8"/>
       <c r="AK8">
         <f t="shared" si="5"/>
@@ -1825,7 +1913,7 @@
       </c>
       <c r="AL8">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM8">
         <f t="shared" si="7"/>
@@ -1849,7 +1937,7 @@
       </c>
       <c r="AS8">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AT8">
         <f t="shared" si="13"/>
@@ -1873,7 +1961,7 @@
       </c>
       <c r="AZ8" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BA8" s="4">
         <f t="shared" si="19"/>
@@ -1894,7 +1982,7 @@
       <c r="BE8" s="4"/>
       <c r="BF8" s="2">
         <f t="shared" si="23"/>
-        <v>1.6833333333333333</v>
+        <v>1.8833333333333333</v>
       </c>
       <c r="BH8">
         <f t="shared" si="24"/>
@@ -1902,7 +1990,7 @@
       </c>
       <c r="BI8">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ8">
         <f t="shared" si="26"/>
@@ -1922,10 +2010,10 @@
       </c>
       <c r="BO8">
         <f t="shared" si="30"/>
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9">
         <f t="shared" si="31"/>
         <v>5</v>
@@ -1987,101 +2075,123 @@
       <c r="V9">
         <v>0</v>
       </c>
-      <c r="W9" s="24"/>
-      <c r="X9"/>
+      <c r="W9" s="24">
+        <v>1</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
       <c r="Y9" s="28">
         <v>0</v>
       </c>
-      <c r="Z9" s="7"/>
-      <c r="AA9" s="35"/>
-      <c r="AB9" s="39"/>
-      <c r="AC9"/>
-      <c r="AD9" s="39"/>
-      <c r="AE9" s="7"/>
-      <c r="AF9" s="24"/>
-      <c r="AG9" s="35"/>
-      <c r="AH9" s="28"/>
+      <c r="Z9" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB9" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC9">
+        <v>2</v>
+      </c>
+      <c r="AD9" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE9" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH9" s="28">
+        <v>1</v>
+      </c>
       <c r="AI9"/>
       <c r="AK9">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL9">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AM9">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AN9">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AO9">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AP9">
         <f t="shared" si="10"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR9">
         <f t="shared" si="11"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AS9">
         <f t="shared" si="12"/>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="AT9">
         <f t="shared" si="13"/>
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="AU9">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AV9">
         <f t="shared" si="15"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="AW9">
         <f t="shared" si="16"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="AY9" s="4">
         <f t="shared" si="17"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AZ9" s="4">
         <f t="shared" si="18"/>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="BA9" s="4">
         <f t="shared" si="19"/>
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="BB9" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BC9" s="4">
         <f t="shared" si="21"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="BD9" s="4">
         <f t="shared" si="22"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="BE9" s="4"/>
       <c r="BF9" s="2">
         <f t="shared" si="23"/>
-        <v>2.5416666666666665</v>
+        <v>4.375</v>
       </c>
       <c r="BH9">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI9">
         <f t="shared" si="25"/>
@@ -2089,26 +2199,26 @@
       </c>
       <c r="BJ9">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK9">
         <f t="shared" si="27"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BL9">
         <f t="shared" si="28"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BM9">
         <f t="shared" si="29"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BO9">
         <f t="shared" si="30"/>
-        <v>3.5</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10">
         <f t="shared" si="31"/>
         <v>6</v>
@@ -2170,40 +2280,62 @@
       <c r="V10">
         <v>2</v>
       </c>
-      <c r="W10" s="24"/>
-      <c r="X10"/>
+      <c r="W10" s="24">
+        <v>1</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
       <c r="Y10" s="28">
         <v>0</v>
       </c>
-      <c r="Z10" s="7"/>
-      <c r="AA10" s="35"/>
-      <c r="AB10" s="39"/>
-      <c r="AC10"/>
-      <c r="AD10" s="39"/>
-      <c r="AE10" s="7"/>
-      <c r="AF10" s="24"/>
-      <c r="AG10" s="35"/>
-      <c r="AH10" s="28"/>
+      <c r="Z10" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB10" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC10">
+        <v>2</v>
+      </c>
+      <c r="AD10" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE10" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="24">
+        <v>1</v>
+      </c>
+      <c r="AG10" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="28">
+        <v>0</v>
+      </c>
       <c r="AI10"/>
       <c r="AK10">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AL10">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AM10">
         <f t="shared" si="7"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AN10">
         <f t="shared" si="8"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AO10">
         <f t="shared" si="9"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AP10">
         <f t="shared" si="10"/>
@@ -2211,23 +2343,23 @@
       </c>
       <c r="AR10">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="AS10">
         <f t="shared" si="12"/>
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="AT10">
         <f t="shared" si="13"/>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="AU10">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AV10">
         <f t="shared" si="15"/>
-        <v>1.3333333333333333</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="AW10">
         <f t="shared" si="16"/>
@@ -2235,23 +2367,23 @@
       </c>
       <c r="AY10" s="4">
         <f t="shared" si="17"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AZ10" s="4">
         <f t="shared" si="18"/>
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="BA10" s="4">
         <f t="shared" si="19"/>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BB10" s="4">
         <f t="shared" si="20"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC10" s="4">
         <f t="shared" si="21"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="BD10" s="4">
         <f t="shared" si="22"/>
@@ -2260,15 +2392,15 @@
       <c r="BE10" s="4"/>
       <c r="BF10" s="2">
         <f t="shared" si="23"/>
-        <v>5.1333333333333329</v>
+        <v>8.5</v>
       </c>
       <c r="BH10">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI10">
         <f t="shared" si="25"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BJ10">
         <f t="shared" si="26"/>
@@ -2276,11 +2408,11 @@
       </c>
       <c r="BK10">
         <f t="shared" si="27"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BL10">
         <f t="shared" si="28"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BM10">
         <f t="shared" si="29"/>
@@ -2288,10 +2420,10 @@
       </c>
       <c r="BO10">
         <f t="shared" si="30"/>
-        <v>6</v>
+        <v>8.5</v>
       </c>
     </row>
-    <row r="11" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11">
         <f t="shared" si="31"/>
         <v>7</v>
@@ -2353,88 +2485,110 @@
       <c r="V11">
         <v>2</v>
       </c>
-      <c r="W11" s="24"/>
-      <c r="X11"/>
+      <c r="W11" s="24">
+        <v>2</v>
+      </c>
+      <c r="X11">
+        <v>2</v>
+      </c>
       <c r="Y11" s="28">
         <v>2</v>
       </c>
-      <c r="Z11" s="7"/>
-      <c r="AA11" s="35"/>
-      <c r="AB11" s="39"/>
-      <c r="AC11"/>
-      <c r="AD11" s="39"/>
-      <c r="AE11" s="7"/>
-      <c r="AF11" s="24"/>
-      <c r="AG11" s="35"/>
-      <c r="AH11" s="28"/>
+      <c r="Z11" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA11" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB11" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC11">
+        <v>2</v>
+      </c>
+      <c r="AD11" s="39">
+        <v>2</v>
+      </c>
+      <c r="AE11" s="7">
+        <v>2</v>
+      </c>
+      <c r="AF11" s="24">
+        <v>2</v>
+      </c>
+      <c r="AG11" s="35">
+        <v>2</v>
+      </c>
+      <c r="AH11" s="28">
+        <v>2</v>
+      </c>
       <c r="AI11"/>
       <c r="AK11">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AL11">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AM11">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AN11">
         <f t="shared" si="8"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AO11">
         <f t="shared" si="9"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AP11">
         <f t="shared" si="10"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AR11">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AS11">
         <f t="shared" si="12"/>
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="AT11">
         <f t="shared" si="13"/>
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="AU11">
         <f t="shared" si="14"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="AV11">
         <f t="shared" si="15"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="AW11">
         <f t="shared" si="16"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="AY11" s="4">
         <f t="shared" si="17"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AZ11" s="4">
         <f t="shared" si="18"/>
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="BA11" s="4">
         <f t="shared" si="19"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BB11" s="4">
         <f t="shared" si="20"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="BC11" s="4">
         <f t="shared" si="21"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="BD11" s="4">
         <f t="shared" si="22"/>
@@ -2443,27 +2597,27 @@
       <c r="BE11" s="4"/>
       <c r="BF11" s="2">
         <f t="shared" si="23"/>
-        <v>6.8666666666666663</v>
+        <v>10</v>
       </c>
       <c r="BH11">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI11">
         <f t="shared" si="25"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BJ11">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK11">
         <f t="shared" si="27"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BL11">
         <f t="shared" si="28"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BM11">
         <f t="shared" si="29"/>
@@ -2471,10 +2625,10 @@
       </c>
       <c r="BO11">
         <f t="shared" si="30"/>
-        <v>7.5</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12">
         <f t="shared" si="31"/>
         <v>8</v>
@@ -2536,97 +2690,119 @@
       <c r="V12">
         <v>0</v>
       </c>
-      <c r="W12" s="24"/>
-      <c r="X12"/>
+      <c r="W12" s="24">
+        <v>1</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
       <c r="Y12" s="28">
         <v>0</v>
       </c>
-      <c r="Z12" s="7"/>
-      <c r="AA12" s="35"/>
-      <c r="AB12" s="39"/>
-      <c r="AC12"/>
-      <c r="AD12" s="39"/>
-      <c r="AE12" s="7"/>
-      <c r="AF12" s="24"/>
-      <c r="AG12" s="35"/>
-      <c r="AH12" s="28"/>
+      <c r="Z12" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="35">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC12">
+        <v>2</v>
+      </c>
+      <c r="AD12" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH12" s="28">
+        <v>2</v>
+      </c>
       <c r="AI12"/>
       <c r="AK12">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL12">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM12">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AN12">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AO12">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP12">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AR12">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AS12">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AT12">
         <f t="shared" si="13"/>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="AU12">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="AV12">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AW12">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AY12" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AZ12" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BA12" s="4">
         <f t="shared" si="19"/>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="BB12" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="BC12" s="4">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="BD12" s="4">
         <f t="shared" si="22"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BE12" s="4"/>
       <c r="BF12" s="2">
         <f t="shared" si="23"/>
-        <v>2.1833333333333336</v>
+        <v>4.5</v>
       </c>
       <c r="BH12">
         <f t="shared" si="24"/>
@@ -2634,7 +2810,7 @@
       </c>
       <c r="BI12">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ12">
         <f t="shared" si="26"/>
@@ -2642,22 +2818,22 @@
       </c>
       <c r="BK12">
         <f t="shared" si="27"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BL12">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BM12">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BO12">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>5.5</v>
       </c>
     </row>
-    <row r="13" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13">
         <f t="shared" si="31"/>
         <v>9</v>
@@ -2719,97 +2895,119 @@
       <c r="V13">
         <v>0</v>
       </c>
-      <c r="W13" s="24"/>
-      <c r="X13"/>
+      <c r="W13" s="24">
+        <v>2</v>
+      </c>
+      <c r="X13">
+        <v>1</v>
+      </c>
       <c r="Y13" s="28">
         <v>2</v>
       </c>
-      <c r="Z13" s="7"/>
-      <c r="AA13" s="35"/>
-      <c r="AB13" s="39"/>
-      <c r="AC13"/>
-      <c r="AD13" s="39"/>
-      <c r="AE13" s="7"/>
-      <c r="AF13" s="24"/>
-      <c r="AG13" s="35"/>
-      <c r="AH13" s="28"/>
+      <c r="Z13" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA13" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB13" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC13">
+        <v>2</v>
+      </c>
+      <c r="AD13" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE13" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG13" s="35">
+        <v>2</v>
+      </c>
+      <c r="AH13" s="28">
+        <v>1</v>
+      </c>
       <c r="AI13"/>
       <c r="AK13">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL13">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM13">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AN13">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AO13">
         <f t="shared" si="9"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AP13">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR13">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AS13">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="AT13">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="AU13">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AV13">
         <f t="shared" si="15"/>
-        <v>0.16666666666666666</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="AW13">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="AY13" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AZ13" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="BA13" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="BB13" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BC13" s="4">
         <f t="shared" si="21"/>
-        <v>0.16666666666666666</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="BD13" s="4">
         <f t="shared" si="22"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="BE13" s="4"/>
       <c r="BF13" s="2">
         <f t="shared" si="23"/>
-        <v>2.0499999999999998</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="BH13">
         <f t="shared" si="24"/>
@@ -2817,30 +3015,30 @@
       </c>
       <c r="BI13">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BJ13">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK13">
         <f t="shared" si="27"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BL13">
         <f t="shared" si="28"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BM13">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BO13">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>5.5</v>
       </c>
     </row>
-    <row r="14" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14">
         <f t="shared" si="31"/>
         <v>10</v>
@@ -2902,20 +3100,42 @@
       <c r="V14">
         <v>0</v>
       </c>
-      <c r="W14" s="24"/>
-      <c r="X14"/>
+      <c r="W14" s="24">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
       <c r="Y14" s="28">
         <v>0</v>
       </c>
-      <c r="Z14" s="7"/>
-      <c r="AA14" s="35"/>
-      <c r="AB14" s="39"/>
-      <c r="AC14"/>
-      <c r="AD14" s="39"/>
-      <c r="AE14" s="7"/>
-      <c r="AF14" s="24"/>
-      <c r="AG14" s="35"/>
-      <c r="AH14" s="28"/>
+      <c r="Z14" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="39">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF14" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="28">
+        <v>0</v>
+      </c>
       <c r="AI14"/>
       <c r="AK14">
         <f t="shared" si="5"/>
@@ -3023,7 +3243,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="15" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15">
         <f t="shared" si="31"/>
         <v>11</v>
@@ -3085,105 +3305,127 @@
       <c r="V15">
         <v>0</v>
       </c>
-      <c r="W15" s="24"/>
-      <c r="X15"/>
+      <c r="W15" s="24">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
       <c r="Y15" s="28">
         <v>0</v>
       </c>
-      <c r="Z15" s="7"/>
-      <c r="AA15" s="35"/>
-      <c r="AB15" s="39"/>
-      <c r="AC15"/>
-      <c r="AD15" s="39"/>
-      <c r="AE15" s="7"/>
-      <c r="AF15" s="24"/>
-      <c r="AG15" s="35"/>
-      <c r="AH15" s="28"/>
+      <c r="Z15" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA15" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB15" s="39">
+        <v>1</v>
+      </c>
+      <c r="AC15">
+        <v>1</v>
+      </c>
+      <c r="AD15" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="24">
+        <v>1</v>
+      </c>
+      <c r="AG15" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH15" s="28">
+        <v>1</v>
+      </c>
       <c r="AI15"/>
       <c r="AK15">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AL15">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM15">
         <f t="shared" si="7"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AN15">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AO15">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AP15">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR15">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="AS15">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AT15">
         <f t="shared" si="13"/>
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="AU15">
         <f t="shared" si="14"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AV15">
         <f t="shared" si="15"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="AW15">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="AY15" s="4">
         <f t="shared" si="17"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AZ15" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BA15" s="4">
         <f t="shared" si="19"/>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BB15" s="4">
         <f t="shared" si="20"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BC15" s="4">
         <f t="shared" si="21"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="BD15" s="4">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BE15" s="4"/>
       <c r="BF15" s="2">
         <f t="shared" si="23"/>
-        <v>2.1</v>
+        <v>3.7833333333333337</v>
       </c>
       <c r="BH15">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BJ15">
         <f t="shared" si="26"/>
@@ -3199,14 +3441,14 @@
       </c>
       <c r="BM15">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BO15">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>4.5</v>
       </c>
     </row>
-    <row r="16" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16">
         <f t="shared" si="31"/>
         <v>12</v>
@@ -3268,109 +3510,131 @@
       <c r="V16">
         <v>2</v>
       </c>
-      <c r="W16" s="24"/>
-      <c r="X16"/>
+      <c r="W16" s="24">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>0</v>
+      </c>
       <c r="Y16" s="28">
         <v>0</v>
       </c>
-      <c r="Z16" s="7"/>
-      <c r="AA16" s="35"/>
-      <c r="AB16" s="39"/>
-      <c r="AC16"/>
-      <c r="AD16" s="39"/>
-      <c r="AE16" s="7"/>
-      <c r="AF16" s="24"/>
-      <c r="AG16" s="35"/>
-      <c r="AH16" s="28"/>
+      <c r="Z16" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA16" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB16" s="39">
+        <v>1</v>
+      </c>
+      <c r="AC16">
+        <v>1</v>
+      </c>
+      <c r="AD16" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF16" s="24">
+        <v>1</v>
+      </c>
+      <c r="AG16" s="35">
+        <v>2</v>
+      </c>
+      <c r="AH16" s="28">
+        <v>2</v>
+      </c>
       <c r="AI16"/>
       <c r="AK16">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL16">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM16">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AN16">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AO16">
         <f t="shared" si="9"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AP16">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AR16">
         <f t="shared" si="11"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AS16">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AT16">
         <f t="shared" si="13"/>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="AU16">
         <f t="shared" si="14"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AV16">
         <f t="shared" si="15"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AW16">
         <f t="shared" si="16"/>
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="AY16" s="4">
         <f t="shared" si="17"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AZ16" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BA16" s="4">
         <f t="shared" si="19"/>
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="BB16" s="4">
         <f t="shared" si="20"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BC16" s="4">
         <f t="shared" si="21"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BD16" s="4">
         <f t="shared" si="22"/>
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="BE16" s="4"/>
       <c r="BF16" s="2">
         <f t="shared" si="23"/>
-        <v>3.2583333333333333</v>
+        <v>5.1416666666666675</v>
       </c>
       <c r="BH16">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI16">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ16">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK16">
         <f t="shared" si="27"/>
@@ -3382,11 +3646,11 @@
       </c>
       <c r="BM16">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BO16">
         <f t="shared" si="30"/>
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="17" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -3451,97 +3715,119 @@
       <c r="V17">
         <v>0</v>
       </c>
-      <c r="W17" s="24"/>
-      <c r="X17"/>
+      <c r="W17" s="24">
+        <v>1</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
       <c r="Y17" s="28">
         <v>0</v>
       </c>
-      <c r="Z17" s="7"/>
-      <c r="AA17" s="35"/>
-      <c r="AB17" s="39"/>
-      <c r="AC17"/>
-      <c r="AD17" s="39"/>
-      <c r="AE17" s="7"/>
-      <c r="AF17" s="24"/>
-      <c r="AG17" s="35"/>
-      <c r="AH17" s="28"/>
+      <c r="Z17" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA17" s="35">
+        <v>1</v>
+      </c>
+      <c r="AB17" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC17">
+        <v>2</v>
+      </c>
+      <c r="AD17" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE17" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF17" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH17" s="28">
+        <v>2</v>
+      </c>
       <c r="AI17"/>
       <c r="AK17">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL17">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM17">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AN17">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AO17">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP17">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AR17">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AS17">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AT17">
         <f t="shared" si="13"/>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="AU17">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AV17">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AW17">
         <f t="shared" si="16"/>
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="AY17" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AZ17" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BA17" s="4">
         <f t="shared" si="19"/>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="BB17" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BC17" s="4">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="BD17" s="4">
         <f t="shared" si="22"/>
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="BE17" s="4"/>
       <c r="BF17" s="2">
         <f t="shared" si="23"/>
-        <v>1.9333333333333333</v>
+        <v>3.916666666666667</v>
       </c>
       <c r="BH17">
         <f t="shared" si="24"/>
@@ -3549,7 +3835,7 @@
       </c>
       <c r="BI17">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ17">
         <f t="shared" si="26"/>
@@ -3557,19 +3843,19 @@
       </c>
       <c r="BK17">
         <f t="shared" si="27"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BL17">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BM17">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BO17">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -3634,101 +3920,123 @@
       <c r="V18">
         <v>2</v>
       </c>
-      <c r="W18" s="24"/>
-      <c r="X18"/>
+      <c r="W18" s="24">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>0</v>
+      </c>
       <c r="Y18" s="28">
         <v>0</v>
       </c>
-      <c r="Z18" s="7"/>
-      <c r="AA18" s="35"/>
-      <c r="AB18" s="39"/>
-      <c r="AC18"/>
-      <c r="AD18" s="39"/>
-      <c r="AE18" s="7"/>
-      <c r="AF18" s="24"/>
-      <c r="AG18" s="35"/>
-      <c r="AH18" s="28"/>
+      <c r="Z18" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA18" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB18" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC18">
+        <v>2</v>
+      </c>
+      <c r="AD18" s="39">
+        <v>2</v>
+      </c>
+      <c r="AE18" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF18" s="24">
+        <v>1</v>
+      </c>
+      <c r="AG18" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH18" s="28">
+        <v>2</v>
+      </c>
       <c r="AI18"/>
       <c r="AK18">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AL18">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AM18">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AN18">
         <f t="shared" si="8"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AO18">
         <f t="shared" si="9"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AP18">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AR18">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.625</v>
       </c>
       <c r="AS18">
         <f t="shared" si="12"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="AT18">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AU18">
         <f t="shared" si="14"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="AV18">
         <f t="shared" si="15"/>
-        <v>1</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="AW18">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AY18" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.625</v>
       </c>
       <c r="AZ18" s="4">
         <f t="shared" si="18"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="BA18" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="BB18" s="4">
         <f t="shared" si="20"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="BC18" s="4">
         <f t="shared" si="21"/>
-        <v>1</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="BD18" s="4">
         <f t="shared" si="22"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BE18" s="4"/>
       <c r="BF18" s="2">
         <f t="shared" si="23"/>
-        <v>4.6833333333333336</v>
+        <v>7.5583333333333327</v>
       </c>
       <c r="BH18">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI18">
         <f t="shared" si="25"/>
@@ -3736,26 +4044,26 @@
       </c>
       <c r="BJ18">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK18">
         <f t="shared" si="27"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BL18">
         <f t="shared" si="28"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BM18">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BO18">
         <f t="shared" si="30"/>
-        <v>5.5</v>
+        <v>8.5</v>
       </c>
     </row>
-    <row r="19" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19">
         <f t="shared" si="31"/>
         <v>15</v>
@@ -3817,24 +4125,46 @@
       <c r="V19">
         <v>0</v>
       </c>
-      <c r="W19" s="24"/>
-      <c r="X19"/>
+      <c r="W19" s="24">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>0</v>
+      </c>
       <c r="Y19" s="28">
         <v>0</v>
       </c>
-      <c r="Z19" s="7"/>
-      <c r="AA19" s="35"/>
-      <c r="AB19" s="39"/>
-      <c r="AC19"/>
-      <c r="AD19" s="39"/>
-      <c r="AE19" s="7"/>
-      <c r="AF19" s="24"/>
-      <c r="AG19" s="35"/>
-      <c r="AH19" s="28"/>
+      <c r="Z19" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA19" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB19" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC19">
+        <v>2</v>
+      </c>
+      <c r="AD19" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE19" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF19" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH19" s="28">
+        <v>0</v>
+      </c>
       <c r="AI19"/>
       <c r="AK19">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AL19">
         <f t="shared" si="6"/>
@@ -3842,15 +4172,15 @@
       </c>
       <c r="AM19">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AN19">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AO19">
         <f t="shared" si="9"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AP19">
         <f t="shared" si="10"/>
@@ -3858,7 +4188,7 @@
       </c>
       <c r="AR19">
         <f t="shared" si="11"/>
-        <v>0.375</v>
+        <v>0.75</v>
       </c>
       <c r="AS19">
         <f t="shared" si="12"/>
@@ -3866,15 +4196,15 @@
       </c>
       <c r="AT19">
         <f t="shared" si="13"/>
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="AU19">
         <f t="shared" si="14"/>
-        <v>0.66666666666666663</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="AV19">
         <f t="shared" si="15"/>
-        <v>0.83333333333333337</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="AW19">
         <f t="shared" si="16"/>
@@ -3882,7 +4212,7 @@
       </c>
       <c r="AY19" s="4">
         <f t="shared" si="17"/>
-        <v>0.375</v>
+        <v>1</v>
       </c>
       <c r="AZ19" s="4">
         <f t="shared" si="18"/>
@@ -3890,15 +4220,15 @@
       </c>
       <c r="BA19" s="4">
         <f t="shared" si="19"/>
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="BB19" s="4">
         <f t="shared" si="20"/>
-        <v>0.66666666666666663</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="BC19" s="4">
         <f t="shared" si="21"/>
-        <v>0.83333333333333337</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="BD19" s="4">
         <f t="shared" si="22"/>
@@ -3907,11 +4237,11 @@
       <c r="BE19" s="4"/>
       <c r="BF19" s="2">
         <f t="shared" si="23"/>
-        <v>3.1750000000000003</v>
+        <v>4.9333333333333336</v>
       </c>
       <c r="BH19">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI19">
         <f t="shared" si="25"/>
@@ -3919,15 +4249,15 @@
       </c>
       <c r="BJ19">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK19">
         <f t="shared" si="27"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BL19">
         <f t="shared" si="28"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BM19">
         <f t="shared" si="29"/>
@@ -3935,10 +4265,10 @@
       </c>
       <c r="BO19">
         <f t="shared" si="30"/>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20">
         <f t="shared" si="31"/>
         <v>16</v>
@@ -4000,97 +4330,119 @@
       <c r="V20">
         <v>0</v>
       </c>
-      <c r="W20" s="24"/>
-      <c r="X20"/>
+      <c r="W20" s="24">
+        <v>1</v>
+      </c>
+      <c r="X20">
+        <v>0</v>
+      </c>
       <c r="Y20" s="28">
         <v>0</v>
       </c>
-      <c r="Z20" s="7"/>
-      <c r="AA20" s="35"/>
-      <c r="AB20" s="39"/>
-      <c r="AC20"/>
-      <c r="AD20" s="39"/>
-      <c r="AE20" s="7"/>
-      <c r="AF20" s="24"/>
-      <c r="AG20" s="35"/>
-      <c r="AH20" s="28"/>
+      <c r="Z20" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA20" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB20" s="39">
+        <v>1</v>
+      </c>
+      <c r="AC20">
+        <v>1</v>
+      </c>
+      <c r="AD20" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH20" s="28">
+        <v>1</v>
+      </c>
       <c r="AI20"/>
       <c r="AK20">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL20">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM20">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AN20">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO20">
         <f t="shared" si="9"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AP20">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR20">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AS20">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AT20">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AU20">
         <f t="shared" si="14"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AV20">
         <f t="shared" si="15"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AW20">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="AY20" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AZ20" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BA20" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="BB20" s="4">
         <f t="shared" si="20"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="BC20" s="4">
         <f t="shared" si="21"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="BD20" s="4">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BE20" s="4"/>
       <c r="BF20" s="2">
         <f t="shared" si="23"/>
-        <v>1.2833333333333334</v>
+        <v>2.6166666666666671</v>
       </c>
       <c r="BH20">
         <f t="shared" si="24"/>
@@ -4098,11 +4450,11 @@
       </c>
       <c r="BI20">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ20">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK20">
         <f t="shared" si="27"/>
@@ -4114,14 +4466,14 @@
       </c>
       <c r="BM20">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BO20">
         <f t="shared" si="30"/>
-        <v>2.5</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21">
         <f t="shared" si="31"/>
         <v>17</v>
@@ -4183,20 +4535,40 @@
       <c r="V21">
         <v>0</v>
       </c>
-      <c r="W21" s="24"/>
-      <c r="X21"/>
+      <c r="W21" s="24">
+        <v>1</v>
+      </c>
+      <c r="X21">
+        <v>0</v>
+      </c>
       <c r="Y21" s="28">
         <v>2</v>
       </c>
-      <c r="Z21" s="7"/>
-      <c r="AA21" s="35"/>
-      <c r="AB21" s="39"/>
+      <c r="Z21" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="39">
+        <v>0</v>
+      </c>
       <c r="AC21"/>
-      <c r="AD21" s="39"/>
-      <c r="AE21" s="7"/>
-      <c r="AF21" s="24"/>
-      <c r="AG21" s="35"/>
-      <c r="AH21" s="28"/>
+      <c r="AD21" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="24">
+        <v>2</v>
+      </c>
+      <c r="AG21" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH21" s="28">
+        <v>2</v>
+      </c>
       <c r="AI21"/>
       <c r="AK21">
         <f t="shared" si="5"/>
@@ -4204,11 +4576,11 @@
       </c>
       <c r="AL21">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AM21">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AN21">
         <f t="shared" si="8"/>
@@ -4220,7 +4592,7 @@
       </c>
       <c r="AP21">
         <f t="shared" si="10"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AR21">
         <f t="shared" si="11"/>
@@ -4228,11 +4600,11 @@
       </c>
       <c r="AS21">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="AT21">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AU21">
         <f t="shared" si="14"/>
@@ -4244,7 +4616,7 @@
       </c>
       <c r="AW21">
         <f t="shared" si="16"/>
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="AY21" s="4">
         <f t="shared" si="17"/>
@@ -4252,11 +4624,11 @@
       </c>
       <c r="AZ21" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="BA21" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="BB21" s="4">
         <f t="shared" si="20"/>
@@ -4268,12 +4640,12 @@
       </c>
       <c r="BD21" s="4">
         <f t="shared" si="22"/>
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="BE21" s="4"/>
       <c r="BF21" s="2">
         <f t="shared" si="23"/>
-        <v>3.5333333333333332</v>
+        <v>4.9833333333333334</v>
       </c>
       <c r="BH21">
         <f t="shared" si="24"/>
@@ -4281,7 +4653,7 @@
       </c>
       <c r="BI21">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ21">
         <f t="shared" si="26"/>
@@ -4297,14 +4669,14 @@
       </c>
       <c r="BM21">
         <f t="shared" si="29"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BO21">
         <f t="shared" si="30"/>
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
-    <row r="22" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22">
         <f t="shared" si="31"/>
         <v>18</v>
@@ -4366,24 +4738,46 @@
       <c r="V22">
         <v>0</v>
       </c>
-      <c r="W22" s="24"/>
-      <c r="X22"/>
+      <c r="W22" s="24">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>0</v>
+      </c>
       <c r="Y22" s="28">
         <v>0</v>
       </c>
-      <c r="Z22" s="7"/>
-      <c r="AA22" s="35"/>
-      <c r="AB22" s="39"/>
-      <c r="AC22"/>
-      <c r="AD22" s="39"/>
-      <c r="AE22" s="7"/>
-      <c r="AF22" s="24"/>
-      <c r="AG22" s="35"/>
-      <c r="AH22" s="28"/>
+      <c r="Z22" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA22" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB22" s="39">
+        <v>1</v>
+      </c>
+      <c r="AC22">
+        <v>1</v>
+      </c>
+      <c r="AD22" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="28">
+        <v>0</v>
+      </c>
       <c r="AI22"/>
       <c r="AK22">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL22">
         <f t="shared" si="6"/>
@@ -4391,15 +4785,15 @@
       </c>
       <c r="AM22">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN22">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO22">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP22">
         <f t="shared" si="10"/>
@@ -4407,7 +4801,7 @@
       </c>
       <c r="AR22">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AS22">
         <f t="shared" si="12"/>
@@ -4415,15 +4809,15 @@
       </c>
       <c r="AT22">
         <f t="shared" si="13"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AU22">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="AV22">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="AW22">
         <f t="shared" si="16"/>
@@ -4431,7 +4825,7 @@
       </c>
       <c r="AY22" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AZ22" s="4">
         <f t="shared" si="18"/>
@@ -4439,15 +4833,15 @@
       </c>
       <c r="BA22" s="4">
         <f t="shared" si="19"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BB22" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="BC22" s="4">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="BD22" s="4">
         <f t="shared" si="22"/>
@@ -4456,7 +4850,7 @@
       <c r="BE22" s="4"/>
       <c r="BF22" s="2">
         <f t="shared" si="23"/>
-        <v>1.8833333333333333</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="BH22">
         <f t="shared" si="24"/>
@@ -4468,7 +4862,7 @@
       </c>
       <c r="BJ22">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK22">
         <f t="shared" si="27"/>
@@ -4476,7 +4870,7 @@
       </c>
       <c r="BL22">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BM22">
         <f t="shared" si="29"/>
@@ -4484,10 +4878,10 @@
       </c>
       <c r="BO22">
         <f t="shared" si="30"/>
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
-    <row r="23" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23">
         <f t="shared" si="31"/>
         <v>19</v>
@@ -4549,20 +4943,42 @@
       <c r="V23">
         <v>0</v>
       </c>
-      <c r="W23" s="24"/>
-      <c r="X23"/>
+      <c r="W23" s="24">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
       <c r="Y23" s="28">
         <v>0</v>
       </c>
-      <c r="Z23" s="7"/>
-      <c r="AA23" s="35"/>
-      <c r="AB23" s="39"/>
-      <c r="AC23"/>
-      <c r="AD23" s="39"/>
-      <c r="AE23" s="7"/>
-      <c r="AF23" s="24"/>
-      <c r="AG23" s="35"/>
-      <c r="AH23" s="28"/>
+      <c r="Z23" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="39">
+        <v>0</v>
+      </c>
+      <c r="AC23">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="28">
+        <v>0</v>
+      </c>
       <c r="AI23"/>
       <c r="AK23">
         <f t="shared" si="5"/>
@@ -4670,7 +5086,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="24" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24">
         <f t="shared" si="31"/>
         <v>20</v>
@@ -4732,20 +5148,42 @@
       <c r="V24">
         <v>0</v>
       </c>
-      <c r="W24" s="24"/>
-      <c r="X24"/>
+      <c r="W24" s="24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
       <c r="Y24" s="28">
         <v>0</v>
       </c>
-      <c r="Z24" s="7"/>
-      <c r="AA24" s="35"/>
-      <c r="AB24" s="39"/>
-      <c r="AC24"/>
-      <c r="AD24" s="39"/>
-      <c r="AE24" s="7"/>
-      <c r="AF24" s="24"/>
-      <c r="AG24" s="35"/>
-      <c r="AH24" s="28"/>
+      <c r="Z24" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC24">
+        <v>2</v>
+      </c>
+      <c r="AD24" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF24" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG24" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="28">
+        <v>0</v>
+      </c>
       <c r="AI24"/>
       <c r="AK24">
         <f t="shared" si="5"/>
@@ -4761,11 +5199,11 @@
       </c>
       <c r="AN24">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AO24">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AP24">
         <f t="shared" si="10"/>
@@ -4785,11 +5223,11 @@
       </c>
       <c r="AU24">
         <f t="shared" si="14"/>
-        <v>0.5</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AV24">
         <f t="shared" si="15"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="AW24">
         <f t="shared" si="16"/>
@@ -4809,11 +5247,11 @@
       </c>
       <c r="BB24" s="4">
         <f t="shared" si="20"/>
-        <v>0.5</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BC24" s="4">
         <f t="shared" si="21"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="BD24" s="4">
         <f t="shared" si="22"/>
@@ -4822,7 +5260,7 @@
       <c r="BE24" s="4"/>
       <c r="BF24" s="2">
         <f t="shared" si="23"/>
-        <v>2.1333333333333333</v>
+        <v>2.8</v>
       </c>
       <c r="BH24">
         <f t="shared" si="24"/>
@@ -4838,11 +5276,11 @@
       </c>
       <c r="BK24">
         <f t="shared" si="27"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BL24">
         <f t="shared" si="28"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BM24">
         <f t="shared" si="29"/>
@@ -4850,10 +5288,10 @@
       </c>
       <c r="BO24">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>59</v>
       </c>
@@ -4911,128 +5349,150 @@
       <c r="V25">
         <v>2</v>
       </c>
-      <c r="W25" s="24"/>
-      <c r="X25"/>
+      <c r="W25" s="24">
+        <v>2</v>
+      </c>
+      <c r="X25">
+        <v>2</v>
+      </c>
       <c r="Y25" s="28">
         <v>2</v>
       </c>
-      <c r="Z25" s="7"/>
-      <c r="AA25" s="35"/>
-      <c r="AB25" s="39"/>
-      <c r="AC25"/>
-      <c r="AD25" s="39"/>
-      <c r="AE25" s="7"/>
-      <c r="AF25" s="24"/>
-      <c r="AG25" s="35"/>
-      <c r="AH25" s="28"/>
+      <c r="Z25" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA25" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB25" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC25">
+        <v>1</v>
+      </c>
+      <c r="AD25" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE25" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="24">
+        <v>2</v>
+      </c>
+      <c r="AG25" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH25" s="28">
+        <v>1</v>
+      </c>
       <c r="AI25"/>
       <c r="AK25">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL25">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AM25">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AN25">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AO25">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AP25">
         <f t="shared" si="10"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR25">
         <f t="shared" si="11"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AS25">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="AT25">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AU25">
         <f t="shared" si="14"/>
-        <v>0.83333333333333337</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="AV25">
         <f t="shared" si="15"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="AW25">
         <f t="shared" si="16"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="AY25" s="4">
         <f t="shared" si="17"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AZ25" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="BA25" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="BB25" s="4">
         <f t="shared" si="20"/>
-        <v>0.83333333333333337</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="BC25" s="4">
         <f t="shared" si="21"/>
-        <v>0.33333333333333331</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="BD25" s="4">
         <f t="shared" si="22"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="BE25" s="4"/>
       <c r="BF25" s="2">
         <f t="shared" si="23"/>
-        <v>2.3416666666666668</v>
+        <v>4.9416666666666664</v>
       </c>
       <c r="BH25">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI25">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ25">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK25">
         <f t="shared" si="27"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BL25">
         <f t="shared" si="28"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BM25">
         <f t="shared" si="29"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BO25">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>6.5</v>
       </c>
     </row>
-    <row r="26" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26">
         <f>A24+1</f>
         <v>21</v>
@@ -5094,40 +5554,62 @@
       <c r="V26">
         <v>2</v>
       </c>
-      <c r="W26" s="24"/>
-      <c r="X26"/>
+      <c r="W26" s="24">
+        <v>2</v>
+      </c>
+      <c r="X26">
+        <v>1</v>
+      </c>
       <c r="Y26" s="28">
         <v>2</v>
       </c>
-      <c r="Z26" s="7"/>
-      <c r="AA26" s="35"/>
-      <c r="AB26" s="39"/>
-      <c r="AC26"/>
-      <c r="AD26" s="39"/>
-      <c r="AE26" s="7"/>
-      <c r="AF26" s="24"/>
-      <c r="AG26" s="35"/>
-      <c r="AH26" s="28"/>
+      <c r="Z26" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA26" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB26" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC26">
+        <v>2</v>
+      </c>
+      <c r="AD26" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="28">
+        <v>0</v>
+      </c>
       <c r="AI26"/>
       <c r="AK26">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AL26">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AM26">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AN26">
         <f t="shared" si="8"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AO26">
         <f t="shared" si="9"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AP26">
         <f t="shared" si="10"/>
@@ -5135,23 +5617,23 @@
       </c>
       <c r="AR26">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="AS26">
         <f t="shared" si="12"/>
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="AT26">
         <f t="shared" si="13"/>
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="AU26">
         <f t="shared" si="14"/>
-        <v>1.3333333333333333</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="AV26">
         <f t="shared" si="15"/>
-        <v>0.66666666666666663</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="AW26">
         <f t="shared" si="16"/>
@@ -5159,23 +5641,23 @@
       </c>
       <c r="AY26" s="4">
         <f t="shared" si="17"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AZ26" s="4">
         <f t="shared" si="18"/>
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="BA26" s="4">
         <f t="shared" si="19"/>
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="BB26" s="4">
         <f t="shared" si="20"/>
-        <v>1.3333333333333333</v>
+        <v>2</v>
       </c>
       <c r="BC26" s="4">
         <f t="shared" si="21"/>
-        <v>0.66666666666666663</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="BD26" s="4">
         <f t="shared" si="22"/>
@@ -5184,27 +5666,27 @@
       <c r="BE26" s="4"/>
       <c r="BF26" s="2">
         <f t="shared" si="23"/>
-        <v>5.8</v>
+        <v>8.0666666666666664</v>
       </c>
       <c r="BH26">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI26">
         <f t="shared" si="25"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BJ26">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK26">
         <f t="shared" si="27"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BL26">
         <f t="shared" si="28"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BM26">
         <f t="shared" si="29"/>
@@ -5212,10 +5694,10 @@
       </c>
       <c r="BO26">
         <f t="shared" si="30"/>
-        <v>6.5</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27">
         <f t="shared" si="31"/>
         <v>22</v>
@@ -5277,20 +5759,42 @@
       <c r="V27">
         <v>0</v>
       </c>
-      <c r="W27" s="24"/>
-      <c r="X27"/>
+      <c r="W27" s="24">
+        <v>0</v>
+      </c>
+      <c r="X27">
+        <v>0</v>
+      </c>
       <c r="Y27" s="28">
         <v>0</v>
       </c>
-      <c r="Z27" s="7"/>
-      <c r="AA27" s="35"/>
-      <c r="AB27" s="39"/>
-      <c r="AC27"/>
-      <c r="AD27" s="39"/>
-      <c r="AE27" s="7"/>
-      <c r="AF27" s="24"/>
-      <c r="AG27" s="35"/>
-      <c r="AH27" s="28"/>
+      <c r="Z27" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="39">
+        <v>1</v>
+      </c>
+      <c r="AC27">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG27" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="28">
+        <v>0</v>
+      </c>
       <c r="AI27"/>
       <c r="AK27">
         <f t="shared" si="5"/>
@@ -5306,7 +5810,7 @@
       </c>
       <c r="AN27">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO27">
         <f t="shared" si="9"/>
@@ -5330,7 +5834,7 @@
       </c>
       <c r="AU27">
         <f t="shared" si="14"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="AV27">
         <f t="shared" si="15"/>
@@ -5354,7 +5858,7 @@
       </c>
       <c r="BB27" s="4">
         <f t="shared" si="20"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="BC27" s="4">
         <f t="shared" si="21"/>
@@ -5367,7 +5871,7 @@
       <c r="BE27" s="4"/>
       <c r="BF27" s="2">
         <f t="shared" si="23"/>
-        <v>2.5083333333333333</v>
+        <v>2.6749999999999998</v>
       </c>
       <c r="BH27">
         <f t="shared" si="24"/>
@@ -5398,7 +5902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:67" ht="17.649999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A28">
         <f t="shared" si="31"/>
         <v>23</v>
@@ -5460,128 +5964,150 @@
       <c r="V28">
         <v>2</v>
       </c>
-      <c r="W28" s="24"/>
-      <c r="X28"/>
+      <c r="W28" s="24">
+        <v>2</v>
+      </c>
+      <c r="X28">
+        <v>1</v>
+      </c>
       <c r="Y28" s="28">
         <v>2</v>
       </c>
-      <c r="Z28" s="7"/>
-      <c r="AA28" s="35"/>
-      <c r="AB28" s="39"/>
-      <c r="AC28"/>
-      <c r="AD28" s="39"/>
-      <c r="AE28" s="7"/>
-      <c r="AF28" s="24"/>
-      <c r="AG28" s="35"/>
-      <c r="AH28" s="28"/>
+      <c r="Z28" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA28" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB28" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC28">
+        <v>2</v>
+      </c>
+      <c r="AD28" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE28" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF28" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG28" s="35">
+        <v>2</v>
+      </c>
+      <c r="AH28" s="28">
+        <v>2</v>
+      </c>
       <c r="AI28"/>
       <c r="AK28">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AL28">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM28">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AN28">
         <f t="shared" si="8"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AO28">
         <f t="shared" si="9"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AP28">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AR28">
         <f t="shared" si="11"/>
-        <v>0.375</v>
+        <v>0.75</v>
       </c>
       <c r="AS28">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="AT28">
         <f t="shared" si="13"/>
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="AU28">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AV28">
         <f t="shared" si="15"/>
-        <v>0.66666666666666663</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="AW28">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AY28" s="4">
         <f t="shared" si="17"/>
-        <v>0.375</v>
+        <v>1</v>
       </c>
       <c r="AZ28" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="BA28" s="4">
         <f t="shared" si="19"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BB28" s="4">
         <f t="shared" si="20"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC28" s="4">
         <f t="shared" si="21"/>
-        <v>0.66666666666666663</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="BD28" s="4">
         <f t="shared" si="22"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BE28" s="4"/>
       <c r="BF28" s="2">
         <f t="shared" si="23"/>
-        <v>3.5416666666666665</v>
+        <v>7.5666666666666673</v>
       </c>
       <c r="BH28">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI28">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BJ28">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK28">
         <f t="shared" si="27"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BL28">
         <f t="shared" si="28"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BM28">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BO28">
         <f t="shared" si="30"/>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:67" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A29">
         <f t="shared" si="31"/>
         <v>24</v>
@@ -5643,24 +6169,46 @@
       <c r="V29">
         <v>2</v>
       </c>
-      <c r="W29" s="24"/>
-      <c r="X29"/>
+      <c r="W29" s="24">
+        <v>0</v>
+      </c>
+      <c r="X29">
+        <v>0</v>
+      </c>
       <c r="Y29" s="28">
         <v>0</v>
       </c>
-      <c r="Z29" s="7"/>
-      <c r="AA29" s="35"/>
-      <c r="AB29" s="39"/>
-      <c r="AC29"/>
-      <c r="AD29" s="39"/>
-      <c r="AE29" s="7"/>
-      <c r="AF29" s="24"/>
-      <c r="AG29" s="35"/>
-      <c r="AH29" s="28"/>
+      <c r="Z29" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA29" s="35">
+        <v>2</v>
+      </c>
+      <c r="AB29" s="39">
+        <v>2</v>
+      </c>
+      <c r="AC29">
+        <v>1</v>
+      </c>
+      <c r="AD29" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="35">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="28">
+        <v>0</v>
+      </c>
       <c r="AI29"/>
       <c r="AK29">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL29">
         <f t="shared" si="6"/>
@@ -5668,15 +6216,15 @@
       </c>
       <c r="AM29">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AN29">
         <f t="shared" si="8"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AO29">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AP29">
         <f t="shared" si="10"/>
@@ -5684,7 +6232,7 @@
       </c>
       <c r="AR29">
         <f t="shared" si="11"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AS29">
         <f t="shared" si="12"/>
@@ -5692,15 +6240,15 @@
       </c>
       <c r="AT29">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AU29">
         <f t="shared" si="14"/>
-        <v>1.1666666666666667</v>
+        <v>1.5</v>
       </c>
       <c r="AV29">
         <f t="shared" si="15"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="AW29">
         <f t="shared" si="16"/>
@@ -5708,7 +6256,7 @@
       </c>
       <c r="AY29" s="4">
         <f t="shared" si="17"/>
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="AZ29" s="4">
         <f t="shared" si="18"/>
@@ -5716,15 +6264,15 @@
       </c>
       <c r="BA29" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="BB29" s="4">
         <f t="shared" si="20"/>
-        <v>1.1666666666666667</v>
+        <v>2</v>
       </c>
       <c r="BC29" s="4">
         <f t="shared" si="21"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="BD29" s="4">
         <f t="shared" si="22"/>
@@ -5733,11 +6281,11 @@
       <c r="BE29" s="4"/>
       <c r="BF29" s="2">
         <f t="shared" si="23"/>
-        <v>3.0750000000000002</v>
+        <v>4.5250000000000004</v>
       </c>
       <c r="BH29">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI29">
         <f t="shared" si="25"/>
@@ -5749,7 +6297,7 @@
       </c>
       <c r="BK29">
         <f t="shared" si="27"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BL29">
         <f t="shared" si="28"/>
@@ -5761,10 +6309,10 @@
       </c>
       <c r="BO29">
         <f t="shared" si="30"/>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:67" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30">
         <f t="shared" si="31"/>
         <v>25</v>
@@ -5826,20 +6374,42 @@
       <c r="V30">
         <v>0</v>
       </c>
-      <c r="W30" s="24"/>
-      <c r="X30"/>
+      <c r="W30" s="24">
+        <v>0</v>
+      </c>
+      <c r="X30">
+        <v>0</v>
+      </c>
       <c r="Y30" s="28">
         <v>0</v>
       </c>
-      <c r="Z30" s="7"/>
-      <c r="AA30" s="35"/>
-      <c r="AB30" s="39"/>
-      <c r="AC30"/>
-      <c r="AD30" s="39"/>
-      <c r="AE30" s="7"/>
-      <c r="AF30" s="24"/>
-      <c r="AG30" s="35"/>
-      <c r="AH30" s="28"/>
+      <c r="Z30" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="35">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="39">
+        <v>0</v>
+      </c>
+      <c r="AC30">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="39">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="24">
+        <v>1</v>
+      </c>
+      <c r="AG30" s="35">
+        <v>1</v>
+      </c>
+      <c r="AH30" s="28">
+        <v>1</v>
+      </c>
       <c r="AI30"/>
       <c r="AK30">
         <f t="shared" si="5"/>
@@ -5847,11 +6417,11 @@
       </c>
       <c r="AL30">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM30">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AN30">
         <f t="shared" si="8"/>
@@ -5863,7 +6433,7 @@
       </c>
       <c r="AP30">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR30">
         <f t="shared" si="11"/>
@@ -5871,11 +6441,11 @@
       </c>
       <c r="AS30">
         <f t="shared" si="12"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="AT30">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AU30">
         <f t="shared" si="14"/>
@@ -5887,7 +6457,7 @@
       </c>
       <c r="AW30">
         <f t="shared" si="16"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="AY30" s="4">
         <f t="shared" si="17"/>
@@ -5895,11 +6465,11 @@
       </c>
       <c r="AZ30" s="4">
         <f t="shared" si="18"/>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="BA30" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="BB30" s="4">
         <f t="shared" si="20"/>
@@ -5911,12 +6481,12 @@
       </c>
       <c r="BD30" s="4">
         <f t="shared" si="22"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="BE30" s="4"/>
       <c r="BF30" s="2">
         <f t="shared" si="23"/>
-        <v>2.1583333333333332</v>
+        <v>2.708333333333333</v>
       </c>
       <c r="BH30">
         <f t="shared" si="24"/>
@@ -5924,7 +6494,7 @@
       </c>
       <c r="BI30">
         <f t="shared" si="25"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BJ30">
         <f t="shared" si="26"/>
@@ -5944,10 +6514,10 @@
       </c>
       <c r="BO30">
         <f t="shared" si="30"/>
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
-    <row r="31" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31">
         <f t="shared" si="31"/>
         <v>26</v>
@@ -6009,85 +6579,118 @@
       <c r="V31" s="19">
         <v>0</v>
       </c>
+      <c r="W31" s="26">
+        <v>0</v>
+      </c>
+      <c r="X31" s="19">
+        <v>0</v>
+      </c>
       <c r="Y31" s="30">
         <v>0</v>
+      </c>
+      <c r="Z31" s="8">
+        <v>2</v>
+      </c>
+      <c r="AA31" s="36">
+        <v>2</v>
+      </c>
+      <c r="AB31" s="41">
+        <v>2</v>
+      </c>
+      <c r="AC31" s="19">
+        <v>2</v>
+      </c>
+      <c r="AD31" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE31" s="8">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="26">
+        <v>2</v>
+      </c>
+      <c r="AG31" s="36">
+        <v>1</v>
+      </c>
+      <c r="AH31" s="30">
+        <v>1</v>
       </c>
       <c r="AK31">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL31">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM31">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AN31">
         <f t="shared" si="8"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AO31">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP31">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR31">
         <f t="shared" si="11"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AS31">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="AT31">
         <f t="shared" si="13"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AU31">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AV31">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="AW31">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="AY31" s="4">
         <f t="shared" si="17"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="AZ31" s="4">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="BA31" s="4">
         <f t="shared" si="19"/>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="BB31" s="4">
         <f t="shared" si="20"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC31" s="4">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="BD31" s="4">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BE31" s="4"/>
       <c r="BF31" s="2">
         <f t="shared" si="23"/>
-        <v>1.55</v>
+        <v>4.0833333333333339</v>
       </c>
       <c r="BH31">
         <f t="shared" si="24"/>
@@ -6095,30 +6698,30 @@
       </c>
       <c r="BI31">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BJ31">
         <f t="shared" si="26"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BK31">
         <f t="shared" si="27"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BL31">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BM31">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="BO31">
         <f t="shared" si="30"/>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32">
         <f t="shared" si="31"/>
         <v>27</v>
@@ -6156,7 +6759,7 @@
       <c r="N32" s="39">
         <v>2</v>
       </c>
-      <c r="O32" s="42">
+      <c r="O32">
         <v>1</v>
       </c>
       <c r="P32" s="21">
@@ -6171,114 +6774,136 @@
       <c r="S32" s="39">
         <v>2</v>
       </c>
-      <c r="T32" s="42">
+      <c r="T32">
         <v>2</v>
       </c>
       <c r="U32" s="39">
         <v>1</v>
       </c>
-      <c r="V32" s="42">
-        <v>2</v>
-      </c>
-      <c r="W32" s="24"/>
-      <c r="X32"/>
+      <c r="V32">
+        <v>2</v>
+      </c>
+      <c r="W32" s="24">
+        <v>2</v>
+      </c>
+      <c r="X32" s="42">
+        <v>2</v>
+      </c>
       <c r="Y32" s="28">
         <v>0</v>
       </c>
-      <c r="Z32" s="7"/>
-      <c r="AA32" s="35"/>
-      <c r="AB32" s="39"/>
-      <c r="AC32"/>
-      <c r="AD32" s="39"/>
-      <c r="AE32" s="7"/>
-      <c r="AF32" s="24"/>
-      <c r="AG32" s="35"/>
-      <c r="AH32" s="28"/>
+      <c r="Z32" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA32" s="35">
+        <v>1</v>
+      </c>
+      <c r="AB32" s="39">
+        <v>0</v>
+      </c>
+      <c r="AC32">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="39">
+        <v>1</v>
+      </c>
+      <c r="AE32" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF32" s="24">
+        <v>1</v>
+      </c>
+      <c r="AG32" s="35">
+        <v>2</v>
+      </c>
+      <c r="AH32" s="28">
+        <v>2</v>
+      </c>
       <c r="AI32"/>
       <c r="AK32">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AL32">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AM32">
         <f t="shared" si="7"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AN32">
         <f t="shared" si="8"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AO32">
         <f t="shared" si="9"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AP32">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AR32">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="AS32">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="AT32">
         <f t="shared" si="13"/>
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="AU32">
         <f t="shared" si="14"/>
-        <v>1.1666666666666667</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="AV32">
         <f t="shared" si="15"/>
-        <v>0.83333333333333337</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="AW32">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="AY32" s="4">
         <f t="shared" si="17"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AZ32" s="4">
         <f t="shared" si="18"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA32" s="4">
         <f t="shared" si="19"/>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BB32" s="4">
         <f t="shared" si="20"/>
-        <v>1.1666666666666667</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="BC32" s="4">
         <f t="shared" si="21"/>
-        <v>0.83333333333333337</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="BD32" s="4">
         <f t="shared" si="22"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BE32" s="4"/>
       <c r="BF32" s="2">
         <f t="shared" si="23"/>
-        <v>5.0999999999999996</v>
+        <v>8.5</v>
       </c>
       <c r="BH32">
         <f t="shared" si="24"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="BI32">
         <f t="shared" si="25"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BJ32">
         <f t="shared" si="26"/>
@@ -6290,15 +6915,15 @@
       </c>
       <c r="BL32">
         <f t="shared" si="28"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="BM32">
         <f t="shared" si="29"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BO32">
         <f t="shared" si="30"/>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="5:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6335,7 +6960,7 @@
       <c r="AI33"/>
       <c r="BO33">
         <f t="shared" ref="BO33" si="32">BO32/2</f>
-        <v>3</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="34" spans="5:67" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -6372,7 +6997,7 @@
       <c r="AI34"/>
       <c r="BO34">
         <f t="shared" ref="BO34" si="33">BO33*100</f>
-        <v>300</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 5f33465 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/CIEL1/CCF/CCF_2025/grille_comp_CCF.xlsx
+++ b/CIEL1/CCF/CCF_2025/grille_comp_CCF.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\CIEL1\CCF\CCF_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7C61D4-F654-4728-91CD-8EBEECA766C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5118CAF-B7A3-4284-80A9-4B84F2DD94C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{5323A597-3EF7-45E9-BE64-C65DC6E6C1EB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{5323A597-3EF7-45E9-BE64-C65DC6E6C1EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -383,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -440,7 +441,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -756,7 +756,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F774E324-096C-456C-BFF9-9E511558E414}">
   <dimension ref="A1:BO34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="6.53125" defaultRowHeight="17.75" customHeight="1" thickBottom="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="6.53125" defaultRowHeight="13.25" customHeight="1" thickBottom="1" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="3" max="3" width="6.53125" style="3"/>
     <col min="4" max="4" width="15.1328125" style="3" customWidth="1"/>
@@ -796,7 +796,7 @@
     <col min="67" max="67" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:67" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B1" t="s">
         <v>29</v>
       </c>
@@ -868,7 +868,7 @@
       <c r="AG1" s="31"/>
       <c r="AI1" s="15"/>
     </row>
-    <row r="2" spans="1:67" s="1" customFormat="1" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:67" s="1" customFormat="1" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B2" s="1" t="s">
         <v>30</v>
       </c>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="D3" s="11"/>
       <c r="E3" s="21" t="s">
         <v>20</v>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="AQ3" s="1"/>
     </row>
-    <row r="4" spans="1:67" ht="17.649999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:67" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="6" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6">
         <f>A5+1</f>
         <v>2</v>
@@ -1603,7 +1603,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="7" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7">
         <f t="shared" ref="A7:A32" si="31">A6+1</f>
         <v>3</v>
@@ -1808,7 +1808,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="8" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8">
         <f t="shared" si="31"/>
         <v>4</v>
@@ -2013,7 +2013,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9">
         <f t="shared" si="31"/>
         <v>5</v>
@@ -2218,7 +2218,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10">
         <f t="shared" si="31"/>
         <v>6</v>
@@ -2423,7 +2423,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="11" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11">
         <f t="shared" si="31"/>
         <v>7</v>
@@ -2628,7 +2628,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12">
         <f t="shared" si="31"/>
         <v>8</v>
@@ -2833,7 +2833,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="13" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13">
         <f t="shared" si="31"/>
         <v>9</v>
@@ -3038,7 +3038,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="14" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14">
         <f t="shared" si="31"/>
         <v>10</v>
@@ -3243,7 +3243,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="15" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15">
         <f t="shared" si="31"/>
         <v>11</v>
@@ -3448,7 +3448,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="16" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16">
         <f t="shared" si="31"/>
         <v>12</v>
@@ -3653,7 +3653,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="17" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17">
         <f t="shared" si="31"/>
         <v>13</v>
@@ -3858,7 +3858,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18">
         <f t="shared" si="31"/>
         <v>14</v>
@@ -4063,7 +4063,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="19" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19">
         <f t="shared" si="31"/>
         <v>15</v>
@@ -4268,7 +4268,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20">
         <f t="shared" si="31"/>
         <v>16</v>
@@ -4473,7 +4473,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21">
         <f t="shared" si="31"/>
         <v>17</v>
@@ -4676,7 +4676,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="22" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22">
         <f t="shared" si="31"/>
         <v>18</v>
@@ -4881,7 +4881,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="23" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23">
         <f t="shared" si="31"/>
         <v>19</v>
@@ -5086,7 +5086,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="24" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24">
         <f t="shared" si="31"/>
         <v>20</v>
@@ -5291,7 +5291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>59</v>
       </c>
@@ -5492,7 +5492,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="26" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26">
         <f>A24+1</f>
         <v>21</v>
@@ -5697,7 +5697,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27">
         <f t="shared" si="31"/>
         <v>22</v>
@@ -5902,7 +5902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:67" ht="17.649999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28">
         <f t="shared" si="31"/>
         <v>23</v>
@@ -6107,7 +6107,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:67" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A29">
         <f t="shared" si="31"/>
         <v>24</v>
@@ -6312,7 +6312,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:67" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30">
         <f t="shared" si="31"/>
         <v>25</v>
@@ -6517,7 +6517,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="31" spans="1:67" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31">
         <f t="shared" si="31"/>
         <v>26</v>
@@ -6721,7 +6721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:67" ht="17.649999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32">
         <f t="shared" si="31"/>
         <v>27</v>
@@ -6786,7 +6786,7 @@
       <c r="W32" s="24">
         <v>2</v>
       </c>
-      <c r="X32" s="42">
+      <c r="X32">
         <v>2</v>
       </c>
       <c r="Y32" s="28">
@@ -6926,7 +6926,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="5:67" ht="17.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="5:67" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="E33" s="7"/>
       <c r="F33" s="35"/>
       <c r="G33" s="24"/>
@@ -6959,11 +6959,11 @@
       <c r="AH33" s="28"/>
       <c r="AI33"/>
       <c r="BO33">
-        <f t="shared" ref="BO33" si="32">BO32/2</f>
-        <v>4.5</v>
+        <f>AVERAGE(BO6:BO32)</f>
+        <v>5.5925925925925926</v>
       </c>
     </row>
-    <row r="34" spans="5:67" ht="17.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="5:67" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="E34" s="7"/>
       <c r="F34" s="35"/>
       <c r="G34" s="24"/>
@@ -6996,8 +6996,8 @@
       <c r="AH34" s="28"/>
       <c r="AI34"/>
       <c r="BO34">
-        <f t="shared" ref="BO34" si="33">BO33*100</f>
-        <v>450</v>
+        <f t="shared" ref="BO34" si="32">BO33*100</f>
+        <v>559.25925925925924</v>
       </c>
     </row>
   </sheetData>
@@ -7005,4 +7005,297 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FCAFC26-A076-4CD2-810F-4F4A63BEC89F}">
+  <dimension ref="A2:B30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="28.53125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="str">
+        <f>Feuil1!B5</f>
+        <v>ACCAR Roger</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="str">
+        <f>Feuil1!B6</f>
+        <v>ADO Oihan</v>
+      </c>
+      <c r="B3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="str">
+        <f>Feuil1!B7</f>
+        <v>ALAUZET Mathis</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="str">
+        <f>Feuil1!B8</f>
+        <v>ARSLANE Djibril</v>
+      </c>
+      <c r="B5">
+        <f>Feuil1!BO8</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="str">
+        <f>Feuil1!B9</f>
+        <v>BENGOUA Solaymane</v>
+      </c>
+      <c r="B6">
+        <f>Feuil1!BO9</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="str">
+        <f>Feuil1!B10</f>
+        <v>BILINGBI MAX Pierre Bradley</v>
+      </c>
+      <c r="B7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" t="str">
+        <f>Feuil1!B11</f>
+        <v>BONVALET icolas</v>
+      </c>
+      <c r="B8">
+        <f>Feuil1!BO11</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" t="str">
+        <f>Feuil1!B12</f>
+        <v>BRENEK Ethan</v>
+      </c>
+      <c r="B9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A10" t="str">
+        <f>Feuil1!B13</f>
+        <v>CHABAUD Nathaniel</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A11" t="str">
+        <f>Feuil1!B14</f>
+        <v>COMBES Sinclair</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A12" t="str">
+        <f>Feuil1!B15</f>
+        <v>EL BOUKHARI Khayfallah</v>
+      </c>
+      <c r="B12">
+        <f>Feuil1!BO15</f>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A13" t="str">
+        <f>Feuil1!B16</f>
+        <v>ELEB Mark</v>
+      </c>
+      <c r="B13">
+        <f>Feuil1!BO16</f>
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A14" t="str">
+        <f>Feuil1!B17</f>
+        <v>FACCINI Adrien</v>
+      </c>
+      <c r="B14">
+        <f>Feuil1!BO17</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A15" t="str">
+        <f>Feuil1!B18</f>
+        <v>FOURCADE Piere</v>
+      </c>
+      <c r="B15">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A16" t="str">
+        <f>Feuil1!B19</f>
+        <v>GIROUD Quentin</v>
+      </c>
+      <c r="B16">
+        <f>Feuil1!BO19</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A17" t="str">
+        <f>Feuil1!B20</f>
+        <v>JABELKHAYR Hatim</v>
+      </c>
+      <c r="B17">
+        <f>Feuil1!BO20</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18" t="str">
+        <f>Feuil1!B21</f>
+        <v>JOUE--CREITER Lukas</v>
+      </c>
+      <c r="B18">
+        <f>Feuil1!BO21</f>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19" t="str">
+        <f>Feuil1!B22</f>
+        <v>JUDE Stephan</v>
+      </c>
+      <c r="B19">
+        <f>Feuil1!BO22</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A20" t="str">
+        <f>Feuil1!B23</f>
+        <v>KADRI Elias</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A21" t="str">
+        <f>Feuil1!B24</f>
+        <v>KHADIRI Abd el Ali</v>
+      </c>
+      <c r="B21">
+        <f>Feuil1!BO24</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A22" t="str">
+        <f>Feuil1!B25</f>
+        <v>MAZABRAUD</v>
+      </c>
+      <c r="B22">
+        <f>Feuil1!BO25</f>
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A23" t="str">
+        <f>Feuil1!B26</f>
+        <v>MORAGLIA Lowan</v>
+      </c>
+      <c r="B23">
+        <f>Feuil1!BO26</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A24" t="str">
+        <f>Feuil1!B27</f>
+        <v>MOREAU Jean</v>
+      </c>
+      <c r="B24">
+        <f>Feuil1!BO27</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A25" t="str">
+        <f>Feuil1!B28</f>
+        <v>NGUEDAM Kiara</v>
+      </c>
+      <c r="B25">
+        <f>Feuil1!BO28</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A26" t="str">
+        <f>Feuil1!B29</f>
+        <v>RIBEIRO Diala</v>
+      </c>
+      <c r="B26">
+        <f>Feuil1!BO29</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A27" t="str">
+        <f>Feuil1!B30</f>
+        <v>RODRIGUES Leandro</v>
+      </c>
+      <c r="B27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A28" t="str">
+        <f>Feuil1!B31</f>
+        <v>SEGUY Axel</v>
+      </c>
+      <c r="B28">
+        <f>Feuil1!BO31</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A29" t="str">
+        <f>Feuil1!B32</f>
+        <v>TRESMONTAN Jordan</v>
+      </c>
+      <c r="B29">
+        <f>Feuil1!BO32</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A30">
+        <f>Feuil1!B33</f>
+        <v>0</v>
+      </c>
+      <c r="B30">
+        <f>AVERAGE(B2:B29)</f>
+        <v>5.6607142857142856</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>